<commit_message>
feat: módulo PIS/COFINS, conciliação de cooperativas CSRF e isolamento de telas
</commit_message>
<xml_diff>
--- a/CONCILIAÇÃO IRRF_CSRF/PCC/relatorio_conferencia_reinf_R-4020_042026_export_1779208964439_RECIFE.xlsx
+++ b/CONCILIAÇÃO IRRF_CSRF/PCC/relatorio_conferencia_reinf_R-4020_042026_export_1779208964439_RECIFE.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://homehealthcaredr-my.sharepoint.com/personal/jackson_junior_homedoctor_com_br/Documents/Documentos/CONCILIAÇÃO IRRF_CSRF/PCC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://homehealthcaredr-my.sharepoint.com/personal/jackson_junior_homedoctor_com_br/Documents/Documentos/Antigravity/Conferência do Faturamento/CONCILIAÇÃO IRRF_CSRF/PCC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{E7B759C5-DAE2-40E4-A434-6B9354213270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABD387B8-6C44-4FEE-8C56-59186197F9A1}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{E7B759C5-DAE2-40E4-A434-6B9354213270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3767EF36-92C7-4418-BE57-E3840F6633E8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>